<commit_message>
Contactos, vetas y modo afloramiento
</commit_message>
<xml_diff>
--- a/examples/ejemplo_volcanosedimentario.xlsx
+++ b/examples/ejemplo_volcanosedimentario.xlsx
@@ -936,7 +936,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>fault</t>
+          <t>sharp</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>gradual</t>
+          <t>fault</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">

</xml_diff>